<commit_message>
feat(audit): complete Item 11 audit, form touch ergonomics, and vocabulary sync
</commit_message>
<xml_diff>
--- a/next-improvements.xlsx
+++ b/next-improvements.xlsx
@@ -2443,11 +2443,19 @@
       </c>
       <c r="D32" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E32" s="29" t="n"/>
-      <c r="F32" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E32" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F32" s="29" t="inlineStr">
+        <is>
+          <t>Verified type=tel on client forms; added inputMode=numeric/decimal across MoneyField, AdjustCreditLimit, RefundPayment, AdjustStock, Expenses, SectionPricing</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="27" t="n">
@@ -2485,11 +2493,19 @@
       </c>
       <c r="D34" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E34" s="29" t="n"/>
-      <c r="F34" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E34" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F34" s="29" t="inlineStr">
+        <is>
+          <t>Verified via automated suites in tier1-features.test.tsx and RecordPaymentModal.test.tsx (accessible name bindings, focus management, keyboard submit)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="27" t="n">
@@ -2506,11 +2522,19 @@
       </c>
       <c r="D35" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E35" s="29" t="n"/>
-      <c r="F35" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F35" s="29" t="inlineStr">
+        <is>
+          <t>Replaced root CURRENT_STATE.md with link to canonical docs/CURRENT_STATE.md updated with 4 Oct verified metrics</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="27" t="n">
@@ -2527,11 +2551,19 @@
       </c>
       <c r="D36" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E36" s="29" t="n"/>
-      <c r="F36" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E36" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F36" s="29" t="inlineStr">
+        <is>
+          <t>completion.mjs reads .pglite-result.json and .test-result.json; check-pglite writes .pglite-result.json; explicit static status reported if not run</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="27" t="n">
@@ -2548,11 +2580,19 @@
       </c>
       <c r="D37" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E37" s="29" t="n"/>
-      <c r="F37" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F37" s="29" t="inlineStr">
+        <is>
+          <t>vitest.config.ts coverage configured for src/lib/**/*.ts, src/actions/**/*.ts, src/modules/**/*.{ts,tsx}; verified with npm run test</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="27" t="n">
@@ -2569,11 +2609,19 @@
       </c>
       <c r="D38" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E38" s="29" t="n"/>
-      <c r="F38" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E38" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F38" s="29" t="inlineStr">
+        <is>
+          <t>Deduplicated in commit 1292efb (0056x3, 0076x2 -&gt; 0073, 0081, 0082); 150 migrations uniquely sequenced</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="27" t="n">
@@ -2590,11 +2638,19 @@
       </c>
       <c r="D39" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E39" s="29" t="n"/>
-      <c r="F39" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F39" s="29" t="inlineStr">
+        <is>
+          <t>Pinned in migration 0149 (search_path = public, pg_temp); definer-hygiene gate in check:pglite verifies 59/59 pinned</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="27" t="n">
@@ -2653,11 +2709,19 @@
       </c>
       <c r="D42" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E42" s="29" t="n"/>
-      <c r="F42" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E42" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F42" s="29" t="inlineStr">
+        <is>
+          <t>Audited offlineQueue.ts: Dexie v1-v3 compound uniqueness, crash recovery, dead-letter max retries 5, Law 3 delete rejection</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="27" t="n">
@@ -2674,11 +2738,19 @@
       </c>
       <c r="D43" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E43" s="29" t="n"/>
-      <c r="F43" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F43" s="29" t="inlineStr">
+        <is>
+          <t>Audited 0133_create_documents_storage_bucket.sql; flagged P1 anon read/write/delete vulnerability for remediation</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="27" t="n">
@@ -2695,11 +2767,19 @@
       </c>
       <c r="D44" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E44" s="29" t="n"/>
-      <c r="F44" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E44" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F44" s="29" t="inlineStr">
+        <is>
+          <t>Audited vite build: two entry points (index.html, marketing.html), vendor chunks, sourcemap: false, 6.9MB font precache</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="27" t="n">
@@ -2716,11 +2796,19 @@
       </c>
       <c r="D45" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E45" s="29" t="n"/>
-      <c r="F45" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E45" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F45" s="29" t="inlineStr">
+        <is>
+          <t>Audited graft/src/lib/booqable and 0040 tables: number collision (B-900), Law 3 deletes, and decoupling strategy</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="27" t="n">
@@ -2737,11 +2825,19 @@
       </c>
       <c r="D46" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E46" s="29" t="n"/>
-      <c r="F46" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E46" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F46" s="29" t="inlineStr">
+        <is>
+          <t>Added §5 Authoritative Domain Glossary to docs/UI_UX_RULES.md</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="27" t="n">
@@ -2758,11 +2854,19 @@
       </c>
       <c r="D47" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E47" s="29" t="n"/>
-      <c r="F47" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E47" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F47" s="29" t="inlineStr">
+        <is>
+          <t>Replaced gear/equipment discrepancies across modals, reports, tools, and dispatch notes</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="27" t="n">
@@ -2779,11 +2883,19 @@
       </c>
       <c r="D48" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E48" s="29" t="n"/>
-      <c r="F48" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E48" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F48" s="29" t="inlineStr">
+        <is>
+          <t>Replaced all 4 window.confirm occurrences with ConfirmDialog in RecordForm.tsx and InternalNotesPage.tsx; added lint gate</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="27" t="n">
@@ -2800,11 +2912,19 @@
       </c>
       <c r="D49" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E49" s="29" t="n"/>
-      <c r="F49" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E49" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F49" s="29" t="inlineStr">
+        <is>
+          <t>Audited 5-slot BottomBar &amp; streamlined MoreSheet navigation; verified in shell.test.tsx</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="27" t="n">

</xml_diff>

<commit_message>
feat(floor-a11y): form auto-labeling, keyboard focus, triage & workbook sync
- Task 31: Auto-label form fields via useId/cloneElement across AddClient, EquipmentShared, and BookingFormWidgets; added explicit aria-labels on floor workspaces, scanners, and modals
- Task 32: Standardized RentalsList row operations to design system Button variants
- Task 33: Enforced 44px minimum control floor target across interactive controls
- Task 34: Added keyboard navigation (role, tabIndex, onKeyDown) across EvidenceThumbnail, PurchaseRequests, TimesheetTab, and Inventory
- Fixed subRentalSubtotalPaisa typing in pricingPipeline and NewRental useMemo deps
- Delivered docs/audit/15_TODO_DECISIONS_TRIAGE.md and docs/audit/16_NEW_RENTAL_DECOMPOSITION_PLAN.md
- Synchronized next-improvements.xlsx (44/49 tasks done, 89.8%) and PROGRESS.md
</commit_message>
<xml_diff>
--- a/next-improvements.xlsx
+++ b/next-improvements.xlsx
@@ -1956,11 +1956,19 @@
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E13" s="26" t="n"/>
-      <c r="F13" s="26" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>Verified against schema_migrations and applied batches via scripts/apply-cutover-remote.mjs</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="16">
       <c r="A14" s="24" t="n">
@@ -1977,11 +1985,19 @@
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E14" s="26" t="n"/>
-      <c r="F14" s="26" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Applied and verified 0125 through 0152 on live Supabase with backup protocol</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="16">
       <c r="A15" s="24" t="n">
@@ -2027,11 +2043,19 @@
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E16" s="26" t="n"/>
-      <c r="F16" s="26" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>Role permissions verified via test-law6-permissions.mjs &amp; floor-lifecycle.test.tsx</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="16">
       <c r="A17" s="24" t="n">
@@ -2048,11 +2072,19 @@
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E17" s="26" t="n"/>
-      <c r="F17" s="26" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>Cutover executed, verified live objects with scripts/probe-cutover-batches.mjs</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="23.85" customHeight="1" s="16">
       <c r="A18" s="24" t="n">
@@ -2380,11 +2412,19 @@
       </c>
       <c r="D29" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E29" s="29" t="n"/>
-      <c r="F29" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F29" s="29" t="inlineStr">
+        <is>
+          <t>Auto-labeled via useId/cloneElement across AddClient, EquipmentShared, BookingFormWidgets, and explicit aria-labels on floor workspaces, scanners, and modals</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="27" t="n">
@@ -2401,11 +2441,19 @@
       </c>
       <c r="D30" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E30" s="29" t="n"/>
-      <c r="F30" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E30" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F30" s="29" t="inlineStr">
+        <is>
+          <t>Standardized RentalsList row actions to design system variants (primary/secondary/outline) via canonical Button component</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="27" t="n">
@@ -2422,11 +2470,19 @@
       </c>
       <c r="D31" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E31" s="29" t="n"/>
-      <c r="F31" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F31" s="29" t="inlineStr">
+        <is>
+          <t>Enforced min-height 44px floor controls across all interactive elements, verified with npm run lint:shell (0 violations across 580 files)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="27" t="n">
@@ -2472,11 +2528,19 @@
       </c>
       <c r="D33" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E33" s="29" t="n"/>
-      <c r="F33" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F33" s="29" t="inlineStr">
+        <is>
+          <t>Added role, tabIndex=0, aria-labels, and onKeyDown keyboard navigation across EvidenceThumbnail, PurchaseRequests, TimesheetTab, Inventory rows, and AddItemPanel</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="27" t="n">
@@ -2941,11 +3005,19 @@
       </c>
       <c r="D50" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E50" s="29" t="n"/>
-      <c r="F50" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E50" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t>Completed architectural audit and subcomponent boundary plan in docs/audit/16_NEW_RENTAL_DECOMPOSITION_PLAN.md</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="27" t="n">
@@ -3004,11 +3076,19 @@
       </c>
       <c r="D53" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E53" s="29" t="n"/>
-      <c r="F53" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F53" s="29" t="inlineStr">
+        <is>
+          <t>Triaged all 232 markers across 6 domains in docs/audit/15_TODO_DECISIONS_TRIAGE.md with safe defaults</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:F28"/>

</xml_diff>

<commit_message>
feat(rentals): complete Item 13 NewRental decomposition and workbook sync
- Decompose monolithic NewRental into RentalLineItemsTree, CrewSection, RentalPricingSection, and RentalFinancialRail
- Wire sub-rentals workflow with custom partners and rates in AddItemPanel
- Fix check constraint booking_lines_manual_item_needs_text across quote bridge and line drafts
- Upgrade InternalNotes dispatch with smart entity lookups, ShiftBriefModal export, and 44px control floor
- Update next-improvements.xlsx Task 51 to Done with 45/49 tasks completed
- Verify full verification gate sequence: typecheck, lint, check:pglite (151/151), check:lifecycle (29/29), check:contrast, lint:shell, and production build
</commit_message>
<xml_diff>
--- a/next-improvements.xlsx
+++ b/next-improvements.xlsx
@@ -3034,11 +3034,19 @@
       </c>
       <c r="D51" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E51" s="29" t="n"/>
-      <c r="F51" s="29" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E51" s="29" t="inlineStr">
+        <is>
+          <t>AI / Babin</t>
+        </is>
+      </c>
+      <c r="F51" s="29" t="inlineStr">
+        <is>
+          <t>Decomposed NewRental into RentalLineItemsTree, CrewSection, RentalPricingSection, RentalFinancialRail; verified via unit tests and e2e safety suite</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="27" t="n">

</xml_diff>